<commit_message>
FARMSTAY Black Garlic Shampoo — 1000 штук вместо 3000
По отдельным позициям даем меньше стандартных 3000: список исключений
задается в OVERRIDES.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014WBQJSibVwnfne7GtvuvQZ
</commit_message>
<xml_diff>
--- a/outputs/Заказ покупателю.xlsx
+++ b/outputs/Заказ покупателю.xlsx
@@ -475,7 +475,7 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>13322529</v>
+        <v>12449745</v>
       </c>
     </row>
     <row r="3">
@@ -495,7 +495,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>30000</v>
+        <v>28000</v>
       </c>
     </row>
     <row r="5">
@@ -535,7 +535,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>-33742</v>
+        <v>-906526</v>
       </c>
     </row>
   </sheetData>
@@ -789,32 +789,32 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>FARMSTAY - Black Garlic Nourishing Shampoo [530ml] / Шампунь-кондиционер 2в1 с экстрактом черного чеснока</t>
+          <t>ETUDE - Baking Powder Crunch Pore Scrub [200ml] / Очищающий скраб для лица с содой</t>
         </is>
       </c>
       <c r="B7" s="4" t="n">
-        <v>3239</v>
+        <v>7279</v>
       </c>
       <c r="C7" s="4" t="n">
         <v>3000</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>436.392</v>
+        <v>397.133</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>1309176</v>
+        <v>1191399</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>239</v>
+        <v>4279</v>
       </c>
       <c r="G7" s="4" t="n">
         <v>0</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>239</v>
+        <v>4279</v>
       </c>
       <c r="I7" s="4" t="n">
-        <v>400</v>
+        <v>1800</v>
       </c>
       <c r="J7" t="n">
         <v>2028</v>
@@ -823,32 +823,32 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ETUDE - Baking Powder Crunch Pore Scrub [200ml] / Очищающий скраб для лица с содой</t>
+          <t>FARMSTAY - Collagen &amp; Hyaluronic Acid All-In One Ampoule [250ml] / Сыворотка с коллагеном и гиалуроновой кислотой</t>
         </is>
       </c>
       <c r="B8" s="4" t="n">
-        <v>7279</v>
+        <v>6179</v>
       </c>
       <c r="C8" s="4" t="n">
         <v>3000</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>397.133</v>
+        <v>382.536</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>1191399</v>
+        <v>1147608</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>4279</v>
+        <v>3179</v>
       </c>
       <c r="G8" s="4" t="n">
         <v>0</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>4279</v>
+        <v>3179</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>1800</v>
+        <v>4000</v>
       </c>
       <c r="J8" t="n">
         <v>2028</v>
@@ -857,32 +857,32 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>FARMSTAY - Collagen &amp; Hyaluronic Acid All-In One Ampoule [250ml] / Сыворотка с коллагеном и гиалуроновой кислотой</t>
+          <t>JIGOTT - Snail Lifting Cream [70ml] / Крем для лица увлажняющий антивозрастной</t>
         </is>
       </c>
       <c r="B9" s="4" t="n">
-        <v>6179</v>
+        <v>7463</v>
       </c>
       <c r="C9" s="4" t="n">
         <v>3000</v>
       </c>
       <c r="D9" s="4" t="n">
-        <v>382.536</v>
+        <v>222.497</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>1147608</v>
+        <v>667491</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>3179</v>
+        <v>4463</v>
       </c>
       <c r="G9" s="4" t="n">
         <v>0</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>3179</v>
+        <v>4463</v>
       </c>
       <c r="I9" s="4" t="n">
-        <v>4000</v>
+        <v>600</v>
       </c>
       <c r="J9" t="n">
         <v>2028</v>
@@ -891,32 +891,32 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>JIGOTT - Snail Lifting Cream [70ml] / Крем для лица увлажняющий антивозрастной</t>
+          <t>ENOUGH - Collagen Moisture Essential Cream [50ml] / Увлажняющий крем для лица с коллагеном</t>
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>7463</v>
+        <v>7340</v>
       </c>
       <c r="C10" s="4" t="n">
         <v>3000</v>
       </c>
       <c r="D10" s="4" t="n">
-        <v>222.497</v>
+        <v>177.43</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>667491</v>
+        <v>532290</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>4463</v>
+        <v>4340</v>
       </c>
       <c r="G10" s="4" t="n">
         <v>0</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>4463</v>
+        <v>4340</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>600</v>
+        <v>2000</v>
       </c>
       <c r="J10" t="n">
         <v>2028</v>
@@ -925,32 +925,32 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ENOUGH - Collagen Moisture Essential Cream [50ml] / Увлажняющий крем для лица с коллагеном</t>
+          <t>FARMSTAY - Black Garlic Nourishing Shampoo [530ml] / Шампунь-кондиционер 2в1 с экстрактом черного чеснока</t>
         </is>
       </c>
       <c r="B11" s="4" t="n">
-        <v>7340</v>
+        <v>3239</v>
       </c>
       <c r="C11" s="4" t="n">
-        <v>3000</v>
+        <v>1000</v>
       </c>
       <c r="D11" s="4" t="n">
-        <v>177.43</v>
+        <v>436.392</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>532290</v>
+        <v>436392</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>4340</v>
+        <v>2239</v>
       </c>
       <c r="G11" s="4" t="n">
         <v>0</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>4340</v>
+        <v>2239</v>
       </c>
       <c r="I11" s="4" t="n">
-        <v>2000</v>
+        <v>400</v>
       </c>
       <c r="J11" t="n">
         <v>2028</v>
@@ -966,20 +966,20 @@
         <v>59244</v>
       </c>
       <c r="C12" s="6" t="n">
-        <v>30000</v>
+        <v>28000</v>
       </c>
       <c r="D12" s="6" t="inlineStr"/>
       <c r="E12" s="6" t="n">
-        <v>13322529</v>
+        <v>12449745</v>
       </c>
       <c r="F12" s="6" t="n">
-        <v>29244</v>
+        <v>31244</v>
       </c>
       <c r="G12" s="6" t="n">
         <v>65028</v>
       </c>
       <c r="H12" s="6" t="n">
-        <v>94272</v>
+        <v>96272</v>
       </c>
       <c r="I12" s="6" t="n">
         <v>12800</v>

</xml_diff>